<commit_message>
Migrate site to signal-and-syntax.com
</commit_message>
<xml_diff>
--- a/metadata/CategoriesAndTags.xlsx
+++ b/metadata/CategoriesAndTags.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tomar\source\repos\technical-blog\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7576891F-BAD7-441B-84A6-12D2E6109011}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C82DA554-E9E0-49B7-BB57-060FF9538D02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" activeTab="1" xr2:uid="{71938F04-02B6-4E0B-A9C3-9D48821FDDCD}"/>
+    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{71938F04-02B6-4E0B-A9C3-9D48821FDDCD}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="1" r:id="rId1"/>
@@ -493,7 +493,6 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}" name="Table2" displayName="Table2" ref="A1:D23" totalsRowShown="0">
   <autoFilter ref="A1:D23" xr:uid="{98231BAD-8D29-4B43-9A96-9A801DC4069B}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D23">
-    <sortCondition ref="A2:A23"/>
     <sortCondition ref="B2:B23"/>
   </sortState>
   <tableColumns count="4">
@@ -867,17 +866,17 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="C2" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="D2" s="2" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
-        <v>https://tomarcher.io/posts/discrete-math-in-large-language-models</v>
+        <v>https://tomarcher.io/posts/birthday-paradox</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -885,59 +884,59 @@
         <v>13</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="C3" t="s">
-        <v>57</v>
+        <v>81</v>
       </c>
       <c r="D3" s="2" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
-        <v>https://tomarcher.io/posts/how-large-language-models-handle-context-windows</v>
+        <v>https://tomarcher.io/posts/discrete-math-in-large-language-models</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="C4" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="D4" s="2" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
-        <v>https://tomarcher.io/posts/how-large-language-models-know-things-they-were-never-taught</v>
+        <v>https://tomarcher.io/posts/edmund-fitzgerald</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="C5" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="D5" s="2" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
-        <v>https://tomarcher.io/posts/how-large-languag-models-learn</v>
+        <v>https://tomarcher.io/posts/five-second-rule</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>9</v>
+        <v>66</v>
       </c>
       <c r="C6" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D6" s="2" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
-        <v>https://tomarcher.io/posts/how-large-languag-models-read-code</v>
+        <v>https://tomarcher.io/posts/hash-collisions</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -945,14 +944,14 @@
         <v>13</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>10</v>
+        <v>56</v>
       </c>
       <c r="C7" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="D7" s="2" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
-        <v>https://tomarcher.io/posts/how-large-languag-models-think</v>
+        <v>https://tomarcher.io/posts/how-large-language-models-handle-context-windows</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -960,14 +959,14 @@
         <v>13</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>61</v>
+        <v>82</v>
       </c>
       <c r="C8" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="D8" s="2" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
-        <v>https://tomarcher.io/posts/how-large-languag-models-tokenize-text</v>
+        <v>https://tomarcher.io/posts/how-large-language-models-know-things-they-were-never-taught</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -975,14 +974,14 @@
         <v>13</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>101</v>
+        <v>36</v>
       </c>
       <c r="C9" t="s">
-        <v>102</v>
-      </c>
-      <c r="D9" s="3" t="str">
-        <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
-        <v>https://tomarcher.io/posts/inside-attention-part-1</v>
+        <v>46</v>
+      </c>
+      <c r="D9" s="2" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
+        <v>https://tomarcher.io/posts/how-large-languag-models-learn</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -990,59 +989,59 @@
         <v>13</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>84</v>
+        <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>85</v>
+        <v>49</v>
       </c>
       <c r="D10" s="2" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
-        <v>https://tomarcher.io/posts/temperature-top-p-creativity-knobs</v>
+        <v>https://tomarcher.io/posts/how-large-languag-models-read-code</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>74</v>
+        <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>73</v>
+        <v>48</v>
       </c>
       <c r="D11" s="2" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
-        <v>https://tomarcher.io/posts/birthday-paradox</v>
+        <v>https://tomarcher.io/posts/how-large-languag-models-think</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>77</v>
+        <v>61</v>
       </c>
       <c r="C12" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="D12" s="2" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
-        <v>https://tomarcher.io/posts/edmund-fitzgerald</v>
+        <v>https://tomarcher.io/posts/how-large-languag-models-tokenize-text</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>47</v>
+        <v>101</v>
       </c>
       <c r="C13" t="s">
-        <v>52</v>
-      </c>
-      <c r="D13" s="2" t="str">
-        <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
-        <v>https://tomarcher.io/posts/five-second-rule</v>
+        <v>102</v>
+      </c>
+      <c r="D13" s="3" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
+        <v>https://tomarcher.io/posts/inside-attention-part-1</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -1062,47 +1061,47 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C15" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="D15" s="2" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
-        <v>https://tomarcher.io/posts/rain-paradox</v>
+        <v>https://tomarcher.io/posts/python-dispatch-maps</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="C16" t="s">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="D16" s="2" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
-        <v>https://tomarcher.io/posts/safe-distance-in-traffic</v>
+        <v>https://tomarcher.io/posts/python-integer-division-and-modulus</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C17" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="D17" s="2" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
-        <v>https://tomarcher.io/posts/thermo-water-energy-balance</v>
+        <v>https://tomarcher.io/posts/python-sympy-vs-numpy</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -1110,89 +1109,89 @@
         <v>11</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C18" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D18" s="2" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
-        <v>https://tomarcher.io/posts/three-d-packing</v>
+        <v>https://tomarcher.io/posts/rain-paradox</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C19" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D19" s="2" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
-        <v>https://tomarcher.io/posts/hash-collisions</v>
+        <v>https://tomarcher.io/posts/safe-distance-in-traffic</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>4</v>
+        <v>84</v>
       </c>
       <c r="C20" t="s">
-        <v>50</v>
+        <v>85</v>
       </c>
       <c r="D20" s="2" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
-        <v>https://tomarcher.io/posts/tfp-chatgpt</v>
+        <v>https://tomarcher.io/posts/temperature-top-p-creativity-knobs</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="C21" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="D21" s="2" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
-        <v>https://tomarcher.io/posts/python-dispatch-maps</v>
+        <v>https://tomarcher.io/posts/tfp-chatgpt</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C22" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="D22" s="2" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
-        <v>https://tomarcher.io/posts/python-integer-division-and-modulus</v>
+        <v>https://tomarcher.io/posts/thermo-water-energy-balance</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>41</v>
+        <v>5</v>
       </c>
       <c r="C23" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="D23" s="2" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://tomarcher.io/posts/",Table2[[#This Row],[Post]]))</f>
-        <v>https://tomarcher.io/posts/python-sympy-vs-numpy</v>
+        <v>https://tomarcher.io/posts/three-d-packing</v>
       </c>
     </row>
   </sheetData>

</xml_diff>